<commit_message>
chg: map case type
</commit_message>
<xml_diff>
--- a/data/Input_BoW_Volume.xlsx
+++ b/data/Input_BoW_Volume.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080"/>
+    <workbookView windowWidth="25600" windowHeight="12080" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="PR" sheetId="1" r:id="rId1"/>
+    <sheet name="Trigger" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="2">
   <si>
     <t>Month</t>
   </si>
@@ -1070,9 +1070,99 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
-  <sheetData/>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="12.5454545454545" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1">
+        <v>46204</v>
+      </c>
+      <c r="B8">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1">
+        <v>46235</v>
+      </c>
+      <c r="B9">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B10">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="1">
+        <v>46296</v>
+      </c>
+      <c r="B11">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="1">
+        <v>46327</v>
+      </c>
+      <c r="B12">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="1">
+        <v>46357</v>
+      </c>
+      <c r="B13">
+        <v>300</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>